<commit_message>
push 1 dt 13.05.2026
</commit_message>
<xml_diff>
--- a/src/test/resources/testdata/RegisterData.xlsx
+++ b/src/test/resources/testdata/RegisterData.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\suada.xhafa\IdeaProjects\NewProject1\src\test\resources\testdata\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A7436E0A-716F-4BE2-A337-7490AF7097C4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7B77075B-7EBE-440A-9E42-7FF42DD2A491}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-6300" yWindow="-16785" windowWidth="23250" windowHeight="12450" xr2:uid="{24422D60-867B-4062-9DF6-FDCAACB4E187}"/>
+    <workbookView xWindow="-11085" yWindow="-20790" windowWidth="23250" windowHeight="17955" xr2:uid="{24422D60-867B-4062-9DF6-FDCAACB4E187}"/>
   </bookViews>
   <sheets>
     <sheet name="Register" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="46" uniqueCount="38">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="57" uniqueCount="40">
   <si>
     <t>testCase</t>
   </si>
@@ -77,9 +77,6 @@
     <t>invalidmail</t>
   </si>
   <si>
-    <t>Invalid email</t>
-  </si>
-  <si>
     <t>TC_REGISTER_003</t>
   </si>
   <si>
@@ -131,9 +128,6 @@
     <t>valid@test.com</t>
   </si>
   <si>
-    <t>Username too long</t>
-  </si>
-  <si>
     <t>TC_REGISTER_008</t>
   </si>
   <si>
@@ -153,6 +147,18 @@
   </si>
   <si>
     <t>user@test.com</t>
+  </si>
+  <si>
+    <t>errorType</t>
+  </si>
+  <si>
+    <t>email address</t>
+  </si>
+  <si>
+    <t>requested format</t>
+  </si>
+  <si>
+    <t>incomplete</t>
   </si>
 </sst>
 </file>
@@ -551,13 +557,19 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8C675AA2-5610-4A1D-8100-035269D20F77}">
-  <dimension ref="A1:F11"/>
-  <sheetFormatPr defaultRowHeight="13.8"/>
+  <dimension ref="A1:G11"/>
+  <sheetFormatPr defaultColWidth="52.19921875" defaultRowHeight="13.8"/>
   <cols>
-    <col min="1" max="1" width="30.59765625" customWidth="1"/>
+    <col min="1" max="1" width="18" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="32.5" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="15" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="11.8984375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="16.296875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="21.59765625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="9.69921875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" ht="41.4">
+    <row r="1" spans="1:7">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -576,8 +588,11 @@
       <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-    </row>
-    <row r="2" spans="1:6" ht="41.4">
+      <c r="G1" s="1" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7">
       <c r="A2" s="2" t="s">
         <v>6</v>
       </c>
@@ -594,8 +609,11 @@
       <c r="F2" s="2" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="3" spans="1:6" ht="41.4">
+      <c r="G2" s="2" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7">
       <c r="A3" s="2" t="s">
         <v>9</v>
       </c>
@@ -611,31 +629,37 @@
       <c r="E3" s="2">
         <v>123456</v>
       </c>
-      <c r="F3" s="2" t="s">
+      <c r="F3" t="s">
+        <v>37</v>
+      </c>
+      <c r="G3" s="2" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7">
+      <c r="A4" s="2" t="s">
         <v>12</v>
-      </c>
-    </row>
-    <row r="4" spans="1:6" ht="41.4">
-      <c r="A4" s="2" t="s">
-        <v>13</v>
       </c>
       <c r="B4" s="2"/>
       <c r="C4" s="2"/>
       <c r="D4" s="2"/>
       <c r="E4" s="2"/>
       <c r="F4" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="G4" s="2" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7">
+      <c r="A5" s="2" t="s">
         <v>14</v>
       </c>
-    </row>
-    <row r="5" spans="1:6" ht="41.4">
-      <c r="A5" s="2" t="s">
+      <c r="B5" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="B5" s="2" t="s">
+      <c r="C5" s="3" t="s">
         <v>16</v>
-      </c>
-      <c r="C5" s="3" t="s">
-        <v>17</v>
       </c>
       <c r="D5" s="2">
         <v>123</v>
@@ -644,38 +668,44 @@
         <v>123</v>
       </c>
       <c r="F5" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="G5" s="2" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7">
+      <c r="A6" s="2" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="6" spans="1:6" ht="41.4">
-      <c r="A6" s="2" t="s">
+      <c r="B6" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="B6" s="2" t="s">
+      <c r="C6" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="C6" s="3" t="s">
+      <c r="D6" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="D6" s="2" t="s">
+      <c r="E6" s="2" t="s">
         <v>22</v>
-      </c>
-      <c r="E6" s="2" t="s">
-        <v>23</v>
       </c>
       <c r="F6" s="2" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="7" spans="1:6" ht="41.4">
+      <c r="G6" s="2" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7">
       <c r="A7" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="B7" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="B7" s="2" t="s">
+      <c r="C7" s="2" t="s">
         <v>25</v>
-      </c>
-      <c r="C7" s="2" t="s">
-        <v>26</v>
       </c>
       <c r="D7" s="2">
         <v>111111</v>
@@ -683,19 +713,22 @@
       <c r="E7" s="2">
         <v>111111</v>
       </c>
-      <c r="F7" s="2" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="8" spans="1:6" ht="69">
+      <c r="F7" t="s">
+        <v>39</v>
+      </c>
+      <c r="G7" s="2" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7">
       <c r="A8" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="B8" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="B8" s="2" t="s">
+      <c r="C8" s="3" t="s">
         <v>28</v>
-      </c>
-      <c r="C8" s="3" t="s">
-        <v>29</v>
       </c>
       <c r="D8" s="2">
         <v>123456</v>
@@ -704,18 +737,21 @@
         <v>123456</v>
       </c>
       <c r="F8" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="G8" s="2" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7">
+      <c r="A9" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="B9" s="2" t="s">
         <v>30</v>
       </c>
-    </row>
-    <row r="9" spans="1:6" ht="41.4">
-      <c r="A9" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="B9" s="2" t="s">
-        <v>32</v>
-      </c>
       <c r="C9" s="3" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="D9" s="2">
         <v>123456</v>
@@ -726,16 +762,19 @@
       <c r="F9" s="2" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="10" spans="1:6" ht="41.4">
+      <c r="G9" s="2" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7">
       <c r="A10" s="2" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="B10" s="2">
         <v>123456</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="D10" s="2" t="s">
         <v>3</v>
@@ -743,24 +782,30 @@
       <c r="E10" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="F10" s="2" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="11" spans="1:6" ht="41.4">
+      <c r="F10" t="s">
+        <v>37</v>
+      </c>
+      <c r="G10" s="2" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7">
       <c r="A11" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="B11" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="C11" s="3" t="s">
         <v>35</v>
-      </c>
-      <c r="B11" s="2" t="s">
-        <v>36</v>
-      </c>
-      <c r="C11" s="3" t="s">
-        <v>37</v>
       </c>
       <c r="D11" s="2"/>
       <c r="E11" s="2"/>
       <c r="F11" s="2" t="s">
-        <v>14</v>
+        <v>13</v>
+      </c>
+      <c r="G11" s="2" t="s">
+        <v>3</v>
       </c>
     </row>
   </sheetData>

</xml_diff>